<commit_message>
cluster_vergleich_5vs5: überarbeite Speicherlogik (NK-Sheets + Namensquelle)
- NK_SOURCES besteht weiter für GEZE (Dieselfloater) und EBM (Surcharges)
- Neu: _NK_GLOB_PATTERNS für HERMA/CHT/Fischerwerke/Groz-Beckert (xlsx-Suche)
- _append_nk_sheet() sucht zuerst NK_SOURCES, dann via glob; überspringt falls
  keine xlsx gefunden (HERMA NK ist .docx, CHT/Fischer kein NK-File vorhanden)
- write_excel() liest Kundennamen aus BI-Spalte 'Name'/'Kunden Name', Fallback
  auf bi_name aus analyse()

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/cluster_vergleich/410844_EBM-Papst_Mulfingen_GmbH___Co__KG_cluster.xlsx
+++ b/output/cluster_vergleich/410844_EBM-Papst_Mulfingen_GmbH___Co__KG_cluster.xlsx
@@ -427,148 +427,154 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:X2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="6" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="9" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
     <col width="9" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Typ</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Abw.Typ</t>
+          <t>Auftrags-Nr</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Cluster Key</t>
+          <t>Kunde</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Bordero</t>
+          <t>Empf.PLZ</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Rech-Nr</t>
+          <t>Vers.PLZ</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Kunde</t>
+          <t>Gew.band</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>KNR</t>
+          <t>Zone</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Versender</t>
+          <t>Basis</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Vers.PLZ</t>
+          <t>Tonnage kg</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Empfänger</t>
+          <t>Soll EUR</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Empf.PLZ</t>
+          <t>Fracht EUR</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Diesel EUR</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Tonnage kg</t>
+          <t>Maut EUR</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>LDM</t>
+          <t>Lademittel</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Stpl</t>
+          <t>Peak EUR</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Gew.band</t>
+          <t>Neben EUR</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Basis</t>
+          <t>EUST Zoll</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Soll EUR</t>
+          <t>Versich.</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Ist EUR</t>
+          <t>NK Summe</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>Erlöse</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>Abw. EUR</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Abw. %</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Periode</t>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Abw. Grund</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cluster_vergleich_5vs5: Filterlogik vor Sampling + Rechnungsnummer im Output
Filter 1 (Null-Erlöse): Entfernt Zeilen mit Erlöse Fracht=0/NaN; PRE-Zeilen
mit Dinas-Daten (nk_fracht befüllt) werden behalten.
Filter 2 (Rechnungsnummer): Entfernt Zeilen ohne/leere/0 Rechnungsnummer.
Beide Filter zeigen per-Kunde Vorher/Nachher-Zählungen.
'Rechnungsnummer' als neue Spalte im Export direkt nach 'Auftragsnummer'.

Effekt: 21.298 → 12.099 (Filter 1) → 9.693 (Filter 2) Zeilen

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/cluster_vergleich/410844_EBM-Papst_Mulfingen_GmbH___Co__KG_cluster.xlsx
+++ b/output/cluster_vergleich/410844_EBM-Papst_Mulfingen_GmbH___Co__KG_cluster.xlsx
@@ -427,33 +427,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="9" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="9" customWidth="1" min="23" max="23"/>
-    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="9" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,110 +470,115 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Rech.-Nr</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Kunde</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Land</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Empf.PLZ</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Vers.PLZ</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Gew.band</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Zone</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Basis</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Tonnage kg</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Soll EUR</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Fracht EUR</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Diesel EUR</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Maut EUR</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Lademittel</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Peak EUR</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Neben EUR</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>EUST Zoll</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Versich.</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>NK Summe</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Erlöse</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Abw. EUR</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Abw. %</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Abw. Grund</t>
         </is>

</xml_diff>